<commit_message>
test jenkins for all browsers in headless config
</commit_message>
<xml_diff>
--- a/src/main/resources/FeatureFiles/.done/ContactUsPage_Edge.xlsx
+++ b/src/main/resources/FeatureFiles/.done/ContactUsPage_Edge.xlsx
@@ -130,9 +130,6 @@
   </si>
   <si>
     <t>waitForPageToRender</t>
-  </si>
-  <si>
-    <t>beforeEach</t>
   </si>
   <si>
     <t>afterEach</t>
@@ -295,6 +292,9 @@
   </si>
   <si>
     <t>openBrowser</t>
+  </si>
+  <si>
+    <t>openHeadlessBrowser</t>
   </si>
 </sst>
 </file>
@@ -690,13 +690,13 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
-        <v>38</v>
+        <v>92</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>34</v>
@@ -733,7 +733,7 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>7</v>
@@ -895,7 +895,7 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>7</v>
@@ -904,18 +904,18 @@
         <v>8</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B25" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>8</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
@@ -931,7 +931,7 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B27" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C27" s="2" t="s">
         <v>11</v>
@@ -953,7 +953,7 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B29" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>12</v>
@@ -975,7 +975,7 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B31" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>13</v>
@@ -1052,23 +1052,23 @@
         <v>6</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="29" x14ac:dyDescent="0.35">
       <c r="B39" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>7</v>
@@ -1077,7 +1077,7 @@
         <v>11</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.35">
@@ -1088,7 +1088,7 @@
         <v>11</v>
       </c>
       <c r="D42" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.35">
@@ -1225,23 +1225,23 @@
         <v>6</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B56" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C56" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D56" s="5" t="s">
         <v>45</v>
-      </c>
-      <c r="D56" s="5" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B58" s="2" t="s">
         <v>7</v>
@@ -1294,7 +1294,7 @@
         <v>12</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.35">
@@ -1305,7 +1305,7 @@
         <v>12</v>
       </c>
       <c r="D63" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.35">
@@ -1398,23 +1398,23 @@
         <v>6</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B73" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D73" s="5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A75" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B75" s="2" t="s">
         <v>7</v>
@@ -1467,7 +1467,7 @@
         <v>12</v>
       </c>
       <c r="D79" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.35">
@@ -1478,7 +1478,7 @@
         <v>12</v>
       </c>
       <c r="D80" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.35">
@@ -1489,7 +1489,7 @@
         <v>13</v>
       </c>
       <c r="D81" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.35">
@@ -1500,7 +1500,7 @@
         <v>13</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.35">
@@ -1571,23 +1571,23 @@
         <v>6</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B90" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C90" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D90" s="5" t="s">
         <v>52</v>
-      </c>
-      <c r="D90" s="5" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A92" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B92" s="2" t="s">
         <v>7</v>
@@ -1640,7 +1640,7 @@
         <v>12</v>
       </c>
       <c r="D96" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.35">
@@ -1651,7 +1651,7 @@
         <v>12</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.35">
@@ -1662,7 +1662,7 @@
         <v>13</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.35">
@@ -1673,7 +1673,7 @@
         <v>13</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.35">
@@ -1733,23 +1733,23 @@
         <v>6</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B106" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C106" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D106" s="5" t="s">
         <v>55</v>
-      </c>
-      <c r="D106" s="5" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A108" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B108" s="2" t="s">
         <v>7</v>
@@ -1802,7 +1802,7 @@
         <v>12</v>
       </c>
       <c r="D112" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.35">
@@ -1813,7 +1813,7 @@
         <v>12</v>
       </c>
       <c r="D113" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.35">
@@ -1824,7 +1824,7 @@
         <v>13</v>
       </c>
       <c r="D114" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.35">
@@ -1835,7 +1835,7 @@
         <v>13</v>
       </c>
       <c r="D115" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.35">
@@ -1895,23 +1895,23 @@
         <v>6</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B122" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D122" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A124" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B124" s="2" t="s">
         <v>7</v>
@@ -1964,7 +1964,7 @@
         <v>12</v>
       </c>
       <c r="D128" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.35">
@@ -1975,7 +1975,7 @@
         <v>12</v>
       </c>
       <c r="D129" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.35">
@@ -1986,7 +1986,7 @@
         <v>13</v>
       </c>
       <c r="D130" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.35">
@@ -1997,7 +1997,7 @@
         <v>13</v>
       </c>
       <c r="D131" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.35">
@@ -2057,23 +2057,23 @@
         <v>6</v>
       </c>
       <c r="C137" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B138" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C138" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D138" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A140" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B140" s="2" t="s">
         <v>7</v>
@@ -2126,7 +2126,7 @@
         <v>12</v>
       </c>
       <c r="D144" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.35">
@@ -2137,7 +2137,7 @@
         <v>12</v>
       </c>
       <c r="D145" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.35">
@@ -2148,7 +2148,7 @@
         <v>13</v>
       </c>
       <c r="D146" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.35">
@@ -2159,7 +2159,7 @@
         <v>13</v>
       </c>
       <c r="D147" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.35">
@@ -2219,23 +2219,23 @@
         <v>6</v>
       </c>
       <c r="C153" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B154" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C154" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D154" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A156" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B156" s="2" t="s">
         <v>7</v>
@@ -2370,23 +2370,23 @@
         <v>6</v>
       </c>
       <c r="C168" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B169" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C169" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D169" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A171" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B171" s="2" t="s">
         <v>7</v>
@@ -2521,23 +2521,23 @@
         <v>6</v>
       </c>
       <c r="C183" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="184" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B184" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C184" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D184" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="186" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A186" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B186" s="2" t="s">
         <v>7</v>
@@ -2634,7 +2634,7 @@
         <v>15</v>
       </c>
       <c r="D194" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="195" spans="1:4" x14ac:dyDescent="0.35">
@@ -2642,7 +2642,7 @@
         <v>6</v>
       </c>
       <c r="C195" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="196" spans="1:4" x14ac:dyDescent="0.35">
@@ -2650,7 +2650,7 @@
         <v>7</v>
       </c>
       <c r="C196" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D196" s="2" t="s">
         <v>31</v>
@@ -2658,13 +2658,13 @@
     </row>
     <row r="197" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B197" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C197" t="s">
+        <v>75</v>
+      </c>
+      <c r="D197" s="2" t="s">
         <v>76</v>
-      </c>
-      <c r="D197" s="2" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="198" spans="1:4" x14ac:dyDescent="0.35">
@@ -2672,21 +2672,21 @@
         <v>7</v>
       </c>
       <c r="C198" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D198" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="199" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B199" s="6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C199" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D199" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="200" spans="1:4" x14ac:dyDescent="0.35">
@@ -2751,7 +2751,7 @@
     </row>
     <row r="207" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A207" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B207" s="2" t="s">
         <v>7</v>
@@ -2848,7 +2848,7 @@
         <v>15</v>
       </c>
       <c r="D215" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="216" spans="1:4" x14ac:dyDescent="0.35">
@@ -2908,23 +2908,23 @@
         <v>6</v>
       </c>
       <c r="C221" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="222" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B222" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C222" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D222" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="224" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A224" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B224" s="2" t="s">
         <v>7</v>
@@ -3021,7 +3021,7 @@
         <v>15</v>
       </c>
       <c r="D232" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="233" spans="2:4" x14ac:dyDescent="0.35">
@@ -3029,7 +3029,7 @@
         <v>6</v>
       </c>
       <c r="C233" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="234" spans="2:4" x14ac:dyDescent="0.35">
@@ -3037,10 +3037,10 @@
         <v>14</v>
       </c>
       <c r="C234" t="s">
+        <v>83</v>
+      </c>
+      <c r="D234" s="2" t="s">
         <v>84</v>
-      </c>
-      <c r="D234" s="2" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="235" spans="2:4" x14ac:dyDescent="0.35">
@@ -3081,7 +3081,7 @@
         <v>6</v>
       </c>
       <c r="C238" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="239" spans="2:4" x14ac:dyDescent="0.35">
@@ -3113,7 +3113,7 @@
     </row>
     <row r="243" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A243" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B243" s="2" t="s">
         <v>7</v>
@@ -3210,7 +3210,7 @@
         <v>15</v>
       </c>
       <c r="D251" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="252" spans="1:4" x14ac:dyDescent="0.35">
@@ -3270,23 +3270,23 @@
         <v>6</v>
       </c>
       <c r="C257" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="258" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B258" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C258" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D258" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="260" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A260" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B260" s="2" t="s">
         <v>7</v>
@@ -3383,7 +3383,7 @@
         <v>15</v>
       </c>
       <c r="D268" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="269" spans="1:4" x14ac:dyDescent="0.35">
@@ -3391,7 +3391,7 @@
         <v>6</v>
       </c>
       <c r="C269" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="270" spans="1:4" x14ac:dyDescent="0.35">
@@ -3399,10 +3399,10 @@
         <v>14</v>
       </c>
       <c r="C270" t="s">
+        <v>83</v>
+      </c>
+      <c r="D270" s="2" t="s">
         <v>84</v>
-      </c>
-      <c r="D270" s="2" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="271" spans="1:4" x14ac:dyDescent="0.35">
@@ -3443,18 +3443,18 @@
         <v>6</v>
       </c>
       <c r="C274" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="275" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B275" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C275" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D275" s="2" t="s">
         <v>90</v>
-      </c>
-      <c r="D275" s="2" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="276" spans="1:4" x14ac:dyDescent="0.35">
@@ -3462,7 +3462,7 @@
         <v>24</v>
       </c>
       <c r="C276" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="277" spans="1:4" x14ac:dyDescent="0.35">
@@ -3494,7 +3494,7 @@
     </row>
     <row r="281" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A281" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B281" s="2" t="s">
         <v>29</v>
@@ -3525,7 +3525,7 @@
     </row>
     <row r="2" spans="1:16384" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>7</v>
@@ -3534,7 +3534,7 @@
         <v>11</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
@@ -36301,7 +36301,7 @@
     </row>
     <row r="4" spans="1:16384" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>7</v>
@@ -36310,7 +36310,7 @@
         <v>11</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>